<commit_message>
fix(locations): keep existing locations on supplier imports
- the Avance import reads the IATA code from an IATA column the Apps
  Script adds, instead of guessing it from the station code, which
  missed every airport with a numeric live code (Athens 022) or a
  non-airport station type (Santorini, Corfu, meet and greet); a sheet
  without the column is refused
- a station matching an existing location by IATA keeps that location's
  name and only fills missing country and city, for every broker:
  production locations are the source of truth, and imports used to
  rename them to the supplier's names
- a new location created with an IATA is marked as an airport
</commit_message>
<xml_diff>
--- a/backend/internal/broker/testdata/avance_stations.xlsx
+++ b/backend/internal/broker/testdata/avance_stations.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://avance1.sharepoint.com/sites/Reservations897/Shared Documents/General/Elite Carss/-----------BACKOFFICE-------------/SALES &amp; MARKETING/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{3776FBB3-5B34-4DA4-801C-9008F33068E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01796555-227D-4A5D-85B3-E5E9F1CD691D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Station" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Station!$A$1:$P$1</definedName>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">Station!$A$1:$P$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="785">
   <si>
     <t>Code</t>
   </si>
@@ -2256,44 +2255,182 @@
   </si>
   <si>
     <t>28.0198497</t>
+  </si>
+  <si>
+    <t>IATA</t>
+  </si>
+  <si>
+    <t>AOK</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>022</t>
+  </si>
+  <si>
+    <t>ATH</t>
+  </si>
+  <si>
+    <t>046</t>
+  </si>
+  <si>
+    <t>AXD</t>
+  </si>
+  <si>
+    <t>CFU1</t>
+  </si>
+  <si>
+    <t>CFU</t>
+  </si>
+  <si>
+    <t>CHQ</t>
+  </si>
+  <si>
+    <t>EFL</t>
+  </si>
+  <si>
+    <t>GPA</t>
+  </si>
+  <si>
+    <t>HER1</t>
+  </si>
+  <si>
+    <t>HER</t>
+  </si>
+  <si>
+    <t>IOA</t>
+  </si>
+  <si>
+    <t>JKH</t>
+  </si>
+  <si>
+    <t>JNX</t>
+  </si>
+  <si>
+    <t>JSY</t>
+  </si>
+  <si>
+    <t>015</t>
+  </si>
+  <si>
+    <t>KLX</t>
+  </si>
+  <si>
+    <t>016</t>
+  </si>
+  <si>
+    <t>KGS</t>
+  </si>
+  <si>
+    <t>KVA</t>
+  </si>
+  <si>
+    <t>LXS</t>
+  </si>
+  <si>
+    <t>025</t>
+  </si>
+  <si>
+    <t>026</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>MLO</t>
+  </si>
+  <si>
+    <t>MJT</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>JMK</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>PAS</t>
+  </si>
+  <si>
+    <t>PVK</t>
+  </si>
+  <si>
+    <t>RHO</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>JTR</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>SMI</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>008</t>
+  </si>
+  <si>
+    <t>029</t>
+  </si>
+  <si>
+    <t>SKG</t>
+  </si>
+  <si>
+    <t>032</t>
+  </si>
+  <si>
+    <t>ZTH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="4">
     <numFmt numFmtId="42" formatCode="_-* #,##0\ &quot;€&quot;_-;\-* #,##0\ &quot;€&quot;_-;_-* &quot;-&quot;\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2321,35 +2458,35 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="Comma" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Comma [0]" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Currency" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Currency [0]" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Comma" xfId="4"/>
+    <cellStyle name="Comma [0]" xfId="5"/>
+    <cellStyle name="Currency" xfId="2"/>
+    <cellStyle name="Currency [0]" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Percent" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2362,7 +2499,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2625,27 +2762,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P91"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="true"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="68.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="255.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="100.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" style="1" width="9"/>
+    <col bestFit="true" customWidth="true" max="2" min="2" style="1" width="41.85546875"/>
+    <col bestFit="true" customWidth="true" max="3" min="3" style="1" width="7.140625"/>
+    <col bestFit="true" customWidth="true" max="4" min="4" style="1" width="17.5703125"/>
+    <col bestFit="true" customWidth="true" max="5" min="5" style="1" width="68.140625"/>
+    <col bestFit="true" customWidth="true" max="6" min="6" style="1" width="24.28515625"/>
+    <col bestFit="true" customWidth="true" max="7" min="7" style="1" width="18.7109375"/>
+    <col bestFit="true" customWidth="true" max="8" min="8" style="1" width="8"/>
+    <col bestFit="true" customWidth="true" max="9" min="9" style="1" width="28"/>
+    <col bestFit="true" customWidth="true" max="10" min="10" style="1" width="13.7109375"/>
+    <col bestFit="true" customWidth="true" max="11" min="11" style="1" width="16.42578125"/>
+    <col bestFit="true" customWidth="true" max="12" min="12" style="1" width="15.85546875"/>
+    <col bestFit="true" customWidth="true" max="13" min="13" style="1" width="255.7109375"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" style="1" width="100.42578125"/>
+    <col bestFit="true" customWidth="true" max="15" min="15" style="1" width="18.28515625"/>
+    <col bestFit="true" customWidth="true" max="16" min="16" style="1" width="19.28515625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="20.1" customHeight="true">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2694,8 +2831,11 @@
       <c r="P1" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q1" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="14.45" customHeight="true">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -2742,7 +2882,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="14.45" customHeight="true">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -2789,7 +2929,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="14.45" customHeight="true">
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
@@ -2836,7 +2976,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="14.45" customHeight="true">
       <c r="A5" s="1" t="s">
         <v>47</v>
       </c>
@@ -2883,7 +3023,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="14.45" customHeight="true">
       <c r="A6" s="1" t="s">
         <v>57</v>
       </c>
@@ -2930,7 +3070,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="14.45" customHeight="true">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -2977,7 +3117,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="14.45" customHeight="true">
       <c r="A8" s="1" t="s">
         <v>70</v>
       </c>
@@ -3026,10 +3166,13 @@
       <c r="P8" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q8" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="14.45" customHeight="true">
       <c r="A9" s="1" t="s">
-        <v>77</v>
+        <v>741</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>76</v>
@@ -3074,9 +3217,9 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="14.45" customHeight="true">
       <c r="A10" s="1" t="s">
-        <v>87</v>
+        <v>742</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>86</v>
@@ -3121,9 +3264,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="14.45" customHeight="true">
       <c r="A11" s="1" t="s">
-        <v>97</v>
+        <v>743</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>95</v>
@@ -3167,10 +3310,13 @@
       <c r="P11" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q11" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="14.45" customHeight="true">
       <c r="A12" s="4" t="s">
-        <v>699</v>
+        <v>745</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>707</v>
@@ -3218,7 +3364,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="14.45" customHeight="true">
       <c r="A13" s="1" t="s">
         <v>107</v>
       </c>
@@ -3264,10 +3410,13 @@
       <c r="P13" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q13" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="14.45" customHeight="true">
       <c r="A14" s="1" t="s">
-        <v>126</v>
+        <v>747</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>116</v>
@@ -3311,8 +3460,11 @@
       <c r="P14" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q14" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="14.45" customHeight="true">
       <c r="A15" s="1" t="s">
         <v>127</v>
       </c>
@@ -3358,8 +3510,11 @@
       <c r="P15" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q15" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="14.45" customHeight="true">
       <c r="A16" s="1" t="s">
         <v>136</v>
       </c>
@@ -3405,8 +3560,11 @@
       <c r="P16" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q16" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="14.45" customHeight="true">
       <c r="A17" s="1" t="s">
         <v>145</v>
       </c>
@@ -3452,8 +3610,11 @@
       <c r="P17" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q17" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="14.45" customHeight="true">
       <c r="A18" s="1" t="s">
         <v>153</v>
       </c>
@@ -3497,7 +3658,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="14.45" customHeight="true">
       <c r="A19" s="1" t="s">
         <v>161</v>
       </c>
@@ -3544,7 +3705,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="14.45" customHeight="true">
       <c r="A20" s="1" t="s">
         <v>170</v>
       </c>
@@ -3591,7 +3752,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="14.45" customHeight="true">
       <c r="A21" s="1" t="s">
         <v>179</v>
       </c>
@@ -3638,7 +3799,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="14.45" customHeight="true">
       <c r="A22" s="1" t="s">
         <v>188</v>
       </c>
@@ -3682,7 +3843,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="14.45" customHeight="true">
       <c r="A23" s="1" t="s">
         <v>197</v>
       </c>
@@ -3726,7 +3887,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="14.45" customHeight="true">
       <c r="A24" s="1" t="s">
         <v>206</v>
       </c>
@@ -3770,9 +3931,9 @@
         <v>214</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="14.45" customHeight="true">
       <c r="A25" s="1" t="s">
-        <v>590</v>
+        <v>752</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>215</v>
@@ -3816,72 +3977,75 @@
       <c r="P25" s="1" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q25" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="14.45" customHeight="true">
       <c r="A26" s="1" t="s">
-        <v>685</v>
+        <v>224</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>686</v>
+        <v>225</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="14.45" customHeight="true">
+      <c r="A27" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>686</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>687</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="J26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>688</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="E27" s="1" t="s">
-        <v>226</v>
+        <v>14</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>18</v>
@@ -3893,42 +4057,45 @@
         <v>0</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>231</v>
+        <v>72</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>232</v>
+        <v>73</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="14.45" customHeight="true">
       <c r="A28" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>14</v>
+        <v>244</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>237</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>18</v>
@@ -3946,42 +4113,42 @@
         <v>239</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>72</v>
+        <v>246</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>73</v>
+        <v>237</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="14.45" customHeight="true">
       <c r="A29" s="1" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>229</v>
+        <v>19</v>
       </c>
       <c r="J29" s="1" t="b">
         <v>0</v>
@@ -3990,45 +4157,33 @@
         <v>716</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="14.45" customHeight="true">
       <c r="A30" s="1" t="s">
-        <v>249</v>
+        <v>689</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>250</v>
+        <v>690</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>703</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J30" s="1" t="b">
         <v>0</v>
@@ -4036,31 +4191,19 @@
       <c r="K30" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="L30" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L30" s="3">
+        <v>306978376753</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="14.45" customHeight="true">
       <c r="A31" s="1" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>15</v>
@@ -4071,22 +4214,34 @@
       <c r="K31" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="L31" s="3">
-        <v>306978376753</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L31" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="14.45" customHeight="true">
       <c r="A32" s="1" t="s">
-        <v>691</v>
+        <v>258</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>692</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>704</v>
+        <v>259</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="J32" s="1" t="b">
         <v>0</v>
@@ -4094,22 +4249,37 @@
       <c r="K32" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="L32" s="3" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L32" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="14.45" customHeight="true">
       <c r="A33" s="1" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>261</v>
@@ -4130,39 +4300,39 @@
         <v>716</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>73</v>
+        <v>271</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="14.45" customHeight="true">
       <c r="A34" s="1" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>269</v>
+        <v>14</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>18</v>
@@ -4177,36 +4347,39 @@
         <v>716</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>261</v>
+        <v>73</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="P34" s="1" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>280</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="14.45" customHeight="true">
       <c r="A35" s="1" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>14</v>
+        <v>283</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>276</v>
@@ -4227,30 +4400,24 @@
         <v>277</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="14.45" customHeight="true">
       <c r="A36" s="1" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>283</v>
+        <v>15</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>284</v>
@@ -4274,36 +4441,42 @@
         <v>277</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="N36" s="1" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O36" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="14.45" customHeight="true">
       <c r="A37" s="1" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>15</v>
+        <v>293</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="H37" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>19</v>
+        <v>229</v>
       </c>
       <c r="J37" s="1" t="b">
         <v>0</v>
@@ -4312,36 +4485,39 @@
         <v>716</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="14.45" customHeight="true">
       <c r="A38" s="1" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>109</v>
+        <v>300</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>294</v>
@@ -4359,36 +4535,36 @@
         <v>716</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="14.45" customHeight="true">
       <c r="A39" s="1" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>300</v>
+        <v>23</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>294</v>
@@ -4397,7 +4573,7 @@
         <v>18</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>229</v>
+        <v>311</v>
       </c>
       <c r="J39" s="1" t="b">
         <v>0</v>
@@ -4406,45 +4582,45 @@
         <v>716</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="N39" s="1" t="s">
         <v>302</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="14.45" customHeight="true">
       <c r="A40" s="1" t="s">
-        <v>307</v>
+        <v>758</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>309</v>
+        <v>14</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>294</v>
+        <v>318</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>311</v>
+        <v>19</v>
       </c>
       <c r="J40" s="1" t="b">
         <v>0</v>
@@ -4453,33 +4629,36 @@
         <v>716</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>295</v>
+        <v>319</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>322</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="14.45" customHeight="true">
       <c r="A41" s="1" t="s">
-        <v>316</v>
+        <v>760</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>14</v>
+        <v>325</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>317</v>
@@ -4503,36 +4682,36 @@
         <v>319</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>278</v>
+        <v>327</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="14.45" customHeight="true">
       <c r="A42" s="1" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>18</v>
@@ -4547,39 +4726,39 @@
         <v>716</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="14.45" customHeight="true">
       <c r="A43" s="1" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>332</v>
+        <v>129</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>18</v>
@@ -4594,39 +4773,42 @@
         <v>716</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>346</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="14.45" customHeight="true">
       <c r="A44" s="1" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>129</v>
+        <v>349</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>18</v>
@@ -4641,39 +4823,36 @@
         <v>716</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="14.45" customHeight="true">
       <c r="A45" s="1" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>349</v>
+        <v>129</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>18</v>
@@ -4688,36 +4867,42 @@
         <v>716</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>353</v>
+        <v>344</v>
+      </c>
+      <c r="N45" s="1" t="s">
+        <v>358</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>362</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="14.45" customHeight="true">
       <c r="A46" s="1" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>129</v>
+        <v>365</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>18</v>
@@ -4732,83 +4917,83 @@
         <v>716</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>344</v>
+        <v>369</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="14.45" customHeight="true">
       <c r="A47" s="1" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>19</v>
+        <v>229</v>
       </c>
       <c r="J47" s="1" t="b">
         <v>0</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>369</v>
+        <v>378</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="14.45" customHeight="true">
       <c r="A48" s="1" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>376</v>
@@ -4826,80 +5011,83 @@
         <v>715</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="14.45" customHeight="true">
       <c r="A49" s="1" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J49" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="M49" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="O49" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="P49" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="14.45" customHeight="true">
+      <c r="A50" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I49" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="J49" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="K49" s="1" t="s">
-        <v>715</v>
-      </c>
-      <c r="L49" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="M49" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="N49" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="O49" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="P49" s="1" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="E50" s="1" t="s">
-        <v>129</v>
+        <v>401</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>393</v>
@@ -4923,42 +5111,42 @@
         <v>395</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" ht="14.45" customHeight="true">
       <c r="A51" s="1" t="s">
-        <v>399</v>
+        <v>764</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>19</v>
+        <v>411</v>
       </c>
       <c r="J51" s="1" t="b">
         <v>0</v>
@@ -4967,45 +5155,45 @@
         <v>716</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>395</v>
+        <v>412</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="14.45" customHeight="true">
       <c r="A52" s="1" t="s">
-        <v>407</v>
+        <v>765</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>408</v>
+        <v>417</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>409</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="H52" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="J52" s="1" t="b">
         <v>0</v>
@@ -5014,36 +5202,36 @@
         <v>716</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="14.45" customHeight="true">
       <c r="A53" s="1" t="s">
-        <v>683</v>
+        <v>766</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>417</v>
+        <v>129</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>418</v>
@@ -5052,7 +5240,7 @@
         <v>18</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>419</v>
+        <v>19</v>
       </c>
       <c r="J53" s="1" t="b">
         <v>0</v>
@@ -5061,27 +5249,30 @@
         <v>716</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>421</v>
+        <v>129</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="P53" s="1" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="14.45" customHeight="true">
       <c r="A54" s="1" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>109</v>
@@ -5090,16 +5281,16 @@
         <v>129</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>418</v>
+        <v>435</v>
       </c>
       <c r="H54" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>19</v>
+        <v>436</v>
       </c>
       <c r="J54" s="1" t="b">
         <v>0</v>
@@ -5108,36 +5299,39 @@
         <v>716</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>428</v>
+        <v>437</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>129</v>
+        <v>344</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="P54" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>439</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="14.45" customHeight="true">
       <c r="A55" s="1" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>109</v>
+        <v>300</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>129</v>
+        <v>442</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>435</v>
@@ -5146,54 +5340,54 @@
         <v>18</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="J55" s="1" t="b">
         <v>0</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>344</v>
+        <v>446</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="P55" s="1" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="14.45" customHeight="true">
       <c r="A56" s="1" t="s">
-        <v>440</v>
+        <v>769</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>300</v>
+        <v>96</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>442</v>
+        <v>129</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>435</v>
+        <v>452</v>
       </c>
       <c r="H56" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="J56" s="1" t="b">
         <v>0</v>
@@ -5202,45 +5396,48 @@
         <v>715</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>446</v>
+        <v>129</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>443</v>
+        <v>455</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>447</v>
+        <v>456</v>
       </c>
       <c r="P56" s="1" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>457</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="14.45" customHeight="true">
       <c r="A57" s="1" t="s">
-        <v>450</v>
+        <v>771</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>129</v>
+        <v>458</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>451</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="H57" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>453</v>
+        <v>19</v>
       </c>
       <c r="J57" s="1" t="b">
         <v>0</v>
@@ -5252,42 +5449,27 @@
         <v>454</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>129</v>
+        <v>461</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="P57" s="1" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" ht="14.45" customHeight="true">
       <c r="A58" s="1" t="s">
-        <v>459</v>
+        <v>693</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>458</v>
+        <v>694</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J58" s="1" t="b">
         <v>0</v>
@@ -5296,30 +5478,39 @@
         <v>715</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="M58" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="N58" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="O58" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="P58" s="1" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="M58" t="s">
+        <v>695</v>
+      </c>
+      <c r="N58" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" ht="14.45" customHeight="true">
       <c r="A59" s="1" t="s">
-        <v>693</v>
+        <v>465</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>694</v>
+        <v>466</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>15</v>
+        <v>117</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="J59" s="1" t="b">
         <v>0</v>
@@ -5328,30 +5519,39 @@
         <v>715</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="M59" t="s">
-        <v>695</v>
-      </c>
-      <c r="N59" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>468</v>
+      </c>
+      <c r="M59" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="N59" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="O59" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="P59" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" ht="14.45" customHeight="true">
       <c r="A60" s="1" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>117</v>
+        <v>23</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>118</v>
+        <v>473</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>467</v>
@@ -5372,42 +5572,42 @@
         <v>468</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>122</v>
+        <v>475</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>123</v>
+        <v>474</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="P60" s="1" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="61" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" ht="14.45" customHeight="true">
       <c r="A61" s="1" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>467</v>
+        <v>482</v>
       </c>
       <c r="H61" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>19</v>
+        <v>229</v>
       </c>
       <c r="J61" s="1" t="b">
         <v>0</v>
@@ -5416,45 +5616,42 @@
         <v>715</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>468</v>
+        <v>483</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="N61" s="1" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="P61" s="1" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="62" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" ht="14.45" customHeight="true">
       <c r="A62" s="1" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>479</v>
+        <v>488</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>480</v>
+        <v>489</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="H62" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>229</v>
+        <v>19</v>
       </c>
       <c r="J62" s="1" t="b">
         <v>0</v>
@@ -5463,36 +5660,30 @@
         <v>715</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="O62" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="P62" s="1" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="63" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" ht="14.45" customHeight="true">
       <c r="A63" s="1" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="H63" s="1" t="s">
         <v>18</v>
@@ -5504,30 +5695,42 @@
         <v>0</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="M63" s="1" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="64" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+      <c r="N63" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="O63" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="P63" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" ht="14.45" customHeight="true">
       <c r="A64" s="1" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>497</v>
+        <v>505</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>498</v>
@@ -5536,89 +5739,92 @@
         <v>18</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>19</v>
+        <v>507</v>
       </c>
       <c r="J64" s="1" t="b">
         <v>0</v>
       </c>
       <c r="K64" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="M64" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="O64" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="P64" s="1" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" ht="14.45" customHeight="true">
+      <c r="A65" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="J65" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="K65" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="L64" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="M64" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="N64" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="O64" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="P64" s="1" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="65" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="D65" s="1" t="s">
+      <c r="L65" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="M65" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N65" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="O65" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="P65" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" ht="14.45" customHeight="true">
+      <c r="A66" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="J65" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>715</v>
-      </c>
-      <c r="L65" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="M65" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="P65" s="1" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="66" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="E66" s="1" t="s">
-        <v>129</v>
+        <v>523</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>515</v>
@@ -5627,7 +5833,7 @@
         <v>18</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>516</v>
+        <v>524</v>
       </c>
       <c r="J66" s="1" t="b">
         <v>0</v>
@@ -5636,45 +5842,45 @@
         <v>716</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="M66" s="1" t="s">
-        <v>129</v>
+        <v>526</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="O66" s="1" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="P66" s="1" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="67" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" ht="14.45" customHeight="true">
       <c r="A67" s="1" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>522</v>
+        <v>530</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>23</v>
+        <v>172</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>523</v>
+        <v>531</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>515</v>
+        <v>533</v>
       </c>
       <c r="H67" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="J67" s="1" t="b">
         <v>0</v>
@@ -5683,45 +5889,45 @@
         <v>716</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>522</v>
+        <v>536</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="P67" s="1" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="68" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="14.45" customHeight="true">
       <c r="A68" s="1" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>172</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>533</v>
+        <v>515</v>
       </c>
       <c r="H68" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>534</v>
+        <v>543</v>
       </c>
       <c r="J68" s="1" t="b">
         <v>0</v>
@@ -5730,45 +5936,42 @@
         <v>716</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="N68" s="1" t="s">
-        <v>536</v>
+        <v>544</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>537</v>
+        <v>545</v>
       </c>
       <c r="P68" s="1" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" ht="14.45" customHeight="true">
       <c r="A69" s="1" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>172</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>541</v>
+        <v>549</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>515</v>
+        <v>533</v>
       </c>
       <c r="H69" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>543</v>
+        <v>534</v>
       </c>
       <c r="J69" s="1" t="b">
         <v>0</v>
@@ -5777,36 +5980,39 @@
         <v>716</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>544</v>
+        <v>551</v>
+      </c>
+      <c r="N69" s="1" t="s">
+        <v>552</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="P69" s="1" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="70" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" ht="14.45" customHeight="true">
       <c r="A70" s="1" t="s">
-        <v>547</v>
+        <v>555</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>548</v>
+        <v>556</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>172</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>533</v>
+        <v>515</v>
       </c>
       <c r="H70" s="1" t="s">
         <v>18</v>
@@ -5821,36 +6027,36 @@
         <v>716</v>
       </c>
       <c r="L70" s="1" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="M70" s="1" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="P70" s="1" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="71" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="14.45" customHeight="true">
       <c r="A71" s="1" t="s">
-        <v>555</v>
+        <v>571</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>556</v>
+        <v>572</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>172</v>
+        <v>23</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>558</v>
+        <v>518</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>515</v>
@@ -5859,7 +6065,7 @@
         <v>18</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="J71" s="1" t="b">
         <v>0</v>
@@ -5868,39 +6074,36 @@
         <v>716</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="M71" s="1" t="s">
-        <v>559</v>
-      </c>
-      <c r="N71" s="1" t="s">
-        <v>560</v>
+        <v>574</v>
       </c>
       <c r="O71" s="1" t="s">
-        <v>561</v>
+        <v>575</v>
       </c>
       <c r="P71" s="1" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" ht="14.45" customHeight="true">
       <c r="A72" s="1" t="s">
-        <v>563</v>
+        <v>577</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>564</v>
+        <v>578</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>172</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>565</v>
+        <v>579</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>566</v>
+        <v>580</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>567</v>
+        <v>533</v>
       </c>
       <c r="H72" s="1" t="s">
         <v>18</v>
@@ -5918,33 +6121,33 @@
         <v>517</v>
       </c>
       <c r="M72" s="1" t="s">
-        <v>568</v>
+        <v>581</v>
       </c>
       <c r="N72" s="1" t="s">
         <v>518</v>
       </c>
       <c r="O72" s="1" t="s">
-        <v>569</v>
+        <v>582</v>
       </c>
       <c r="P72" s="1" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" ht="14.45" customHeight="true">
       <c r="A73" s="1" t="s">
-        <v>571</v>
+        <v>584</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>572</v>
+        <v>585</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>573</v>
+        <v>586</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>518</v>
+        <v>587</v>
       </c>
       <c r="G73" s="1" t="s">
         <v>515</v>
@@ -5953,7 +6156,7 @@
         <v>18</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>524</v>
+        <v>19</v>
       </c>
       <c r="J73" s="1" t="b">
         <v>0</v>
@@ -5962,36 +6165,33 @@
         <v>716</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="M73" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="O73" s="1" t="s">
-        <v>575</v>
-      </c>
-      <c r="P73" s="1" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="74" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>588</v>
+      </c>
+      <c r="N73" s="1" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" ht="14.45" customHeight="true">
       <c r="A74" s="1" t="s">
-        <v>577</v>
+        <v>718</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>578</v>
+        <v>719</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>172</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>579</v>
+        <v>720</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>580</v>
+        <v>721</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>533</v>
+        <v>515</v>
       </c>
       <c r="H74" s="1" t="s">
         <v>18</v>
@@ -6009,42 +6209,39 @@
         <v>517</v>
       </c>
       <c r="M74" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="N74" s="1" t="s">
-        <v>518</v>
+        <v>722</v>
       </c>
       <c r="O74" s="1" t="s">
-        <v>582</v>
+        <v>723</v>
       </c>
       <c r="P74" s="1" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="75" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" ht="14.45" customHeight="true">
       <c r="A75" s="1" t="s">
-        <v>584</v>
+        <v>725</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>585</v>
+        <v>726</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>586</v>
+        <v>727</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>587</v>
+        <v>728</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>515</v>
+        <v>567</v>
       </c>
       <c r="H75" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>19</v>
+        <v>534</v>
       </c>
       <c r="J75" s="1" t="b">
         <v>0</v>
@@ -6053,33 +6250,36 @@
         <v>716</v>
       </c>
       <c r="L75" s="1" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="M75" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="N75" s="1" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>729</v>
+      </c>
+      <c r="O75" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="P75" s="1" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" ht="14.45" customHeight="true">
       <c r="A76" s="1" t="s">
-        <v>718</v>
+        <v>732</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>719</v>
+        <v>733</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>172</v>
+        <v>23</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>720</v>
+        <v>734</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>515</v>
+        <v>533</v>
       </c>
       <c r="H76" s="1" t="s">
         <v>18</v>
@@ -6097,39 +6297,39 @@
         <v>517</v>
       </c>
       <c r="M76" s="1" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="O76" s="1" t="s">
-        <v>723</v>
+        <v>737</v>
       </c>
       <c r="P76" s="1" t="s">
-        <v>724</v>
-      </c>
-    </row>
-    <row r="77" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" ht="14.45" customHeight="true">
       <c r="A77" s="1" t="s">
-        <v>725</v>
+        <v>591</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>726</v>
+        <v>592</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>727</v>
+        <v>593</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>728</v>
+        <v>594</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>567</v>
+        <v>595</v>
       </c>
       <c r="H77" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I77" s="1" t="s">
-        <v>534</v>
+        <v>19</v>
       </c>
       <c r="J77" s="1" t="b">
         <v>0</v>
@@ -6138,42 +6338,45 @@
         <v>716</v>
       </c>
       <c r="L77" s="1" t="s">
-        <v>517</v>
+        <v>596</v>
       </c>
       <c r="M77" s="1" t="s">
-        <v>729</v>
+        <v>597</v>
+      </c>
+      <c r="N77" s="1" t="s">
+        <v>594</v>
       </c>
       <c r="O77" s="1" t="s">
-        <v>730</v>
+        <v>598</v>
       </c>
       <c r="P77" s="1" t="s">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="78" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" ht="14.45" customHeight="true">
       <c r="A78" s="1" t="s">
-        <v>732</v>
+        <v>775</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>733</v>
+        <v>600</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>734</v>
+        <v>129</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>735</v>
+        <v>602</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>533</v>
+        <v>603</v>
       </c>
       <c r="H78" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I78" s="1" t="s">
-        <v>534</v>
+        <v>19</v>
       </c>
       <c r="J78" s="1" t="b">
         <v>0</v>
@@ -6182,36 +6385,42 @@
         <v>716</v>
       </c>
       <c r="L78" s="1" t="s">
-        <v>517</v>
+        <v>604</v>
       </c>
       <c r="M78" s="1" t="s">
-        <v>736</v>
+        <v>129</v>
+      </c>
+      <c r="N78" s="1" t="s">
+        <v>605</v>
       </c>
       <c r="O78" s="1" t="s">
-        <v>737</v>
+        <v>606</v>
       </c>
       <c r="P78" s="1" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="79" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>607</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" ht="14.45" customHeight="true">
       <c r="A79" s="1" t="s">
-        <v>591</v>
+        <v>777</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>592</v>
+        <v>608</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>593</v>
+        <v>609</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="H79" s="1" t="s">
         <v>18</v>
@@ -6226,39 +6435,39 @@
         <v>716</v>
       </c>
       <c r="L79" s="1" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="M79" s="1" t="s">
-        <v>597</v>
+        <v>610</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="O79" s="1" t="s">
-        <v>598</v>
+        <v>611</v>
       </c>
       <c r="P79" s="1" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="80" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" ht="14.45" customHeight="true">
       <c r="A80" s="1" t="s">
-        <v>601</v>
+        <v>613</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>23</v>
+        <v>300</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>129</v>
+        <v>615</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>602</v>
+        <v>616</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="H80" s="1" t="s">
         <v>18</v>
@@ -6273,39 +6482,39 @@
         <v>716</v>
       </c>
       <c r="L80" s="1" t="s">
-        <v>604</v>
+        <v>618</v>
       </c>
       <c r="M80" s="1" t="s">
-        <v>129</v>
+        <v>619</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>605</v>
+        <v>620</v>
       </c>
       <c r="O80" s="1" t="s">
-        <v>606</v>
+        <v>621</v>
       </c>
       <c r="P80" s="1" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="81" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" ht="14.45" customHeight="true">
       <c r="A81" s="1" t="s">
-        <v>684</v>
+        <v>623</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>608</v>
+        <v>624</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>609</v>
+        <v>625</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>602</v>
+        <v>624</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>603</v>
+        <v>626</v>
       </c>
       <c r="H81" s="1" t="s">
         <v>18</v>
@@ -6320,39 +6529,42 @@
         <v>716</v>
       </c>
       <c r="L81" s="1" t="s">
-        <v>604</v>
+        <v>627</v>
       </c>
       <c r="M81" s="1" t="s">
-        <v>610</v>
-      </c>
-      <c r="N81" s="1" t="s">
-        <v>602</v>
+        <v>628</v>
       </c>
       <c r="O81" s="1" t="s">
-        <v>611</v>
+        <v>629</v>
       </c>
       <c r="P81" s="1" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="82" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>630</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" ht="14.45" customHeight="true">
       <c r="A82" s="1" t="s">
-        <v>613</v>
+        <v>631</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>614</v>
+        <v>632</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>706</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>300</v>
+        <v>14</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>615</v>
+        <v>67</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>616</v>
+        <v>632</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>617</v>
+        <v>626</v>
       </c>
       <c r="H82" s="1" t="s">
         <v>18</v>
@@ -6367,36 +6579,30 @@
         <v>716</v>
       </c>
       <c r="L82" s="1" t="s">
-        <v>618</v>
+        <v>633</v>
       </c>
       <c r="M82" s="1" t="s">
-        <v>619</v>
+        <v>29</v>
       </c>
       <c r="N82" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="O82" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="P82" s="1" t="s">
-        <v>622</v>
-      </c>
-    </row>
-    <row r="83" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" ht="14.45" customHeight="true">
       <c r="A83" s="1" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>626</v>
@@ -6417,36 +6623,36 @@
         <v>627</v>
       </c>
       <c r="M83" s="1" t="s">
-        <v>628</v>
+        <v>637</v>
+      </c>
+      <c r="N83" s="1" t="s">
+        <v>635</v>
       </c>
       <c r="O83" s="1" t="s">
-        <v>629</v>
+        <v>638</v>
       </c>
       <c r="P83" s="1" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="84" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" ht="14.45" customHeight="true">
       <c r="A84" s="1" t="s">
-        <v>631</v>
+        <v>779</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>632</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>706</v>
+        <v>640</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>67</v>
+        <v>642</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>626</v>
+        <v>644</v>
       </c>
       <c r="H84" s="1" t="s">
         <v>18</v>
@@ -6461,33 +6667,39 @@
         <v>716</v>
       </c>
       <c r="L84" s="1" t="s">
-        <v>633</v>
+        <v>645</v>
       </c>
       <c r="M84" s="1" t="s">
-        <v>29</v>
+        <v>646</v>
       </c>
       <c r="N84" s="1" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="85" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+      <c r="O84" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="P84" s="1" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" ht="14.45" customHeight="true">
       <c r="A85" s="1" t="s">
-        <v>634</v>
+        <v>780</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>635</v>
+        <v>650</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>636</v>
+        <v>652</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>626</v>
+        <v>653</v>
       </c>
       <c r="H85" s="1" t="s">
         <v>18</v>
@@ -6502,45 +6714,45 @@
         <v>716</v>
       </c>
       <c r="L85" s="1" t="s">
-        <v>627</v>
+        <v>654</v>
       </c>
       <c r="M85" s="1" t="s">
-        <v>637</v>
+        <v>655</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>635</v>
+        <v>647</v>
       </c>
       <c r="O85" s="1" t="s">
-        <v>638</v>
+        <v>656</v>
       </c>
       <c r="P85" s="1" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="86" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" ht="14.45" customHeight="true">
       <c r="A86" s="1" t="s">
-        <v>641</v>
+        <v>781</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>640</v>
+        <v>659</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>642</v>
+        <v>129</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>644</v>
+        <v>661</v>
       </c>
       <c r="H86" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>19</v>
+        <v>516</v>
       </c>
       <c r="J86" s="1" t="b">
         <v>0</v>
@@ -6552,42 +6764,27 @@
         <v>645</v>
       </c>
       <c r="M86" s="1" t="s">
-        <v>646</v>
+        <v>662</v>
       </c>
       <c r="N86" s="1" t="s">
         <v>647</v>
       </c>
-      <c r="O86" s="1" t="s">
-        <v>648</v>
-      </c>
-      <c r="P86" s="1" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="87" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q86" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" ht="14.45" customHeight="true">
       <c r="A87" s="1" t="s">
-        <v>651</v>
+        <v>698</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>650</v>
+        <v>697</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>705</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>652</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>643</v>
-      </c>
-      <c r="G87" s="1" t="s">
-        <v>653</v>
-      </c>
-      <c r="H87" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I87" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J87" s="1" t="b">
         <v>0</v>
@@ -6595,46 +6792,31 @@
       <c r="K87" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="L87" s="1" t="s">
-        <v>654</v>
-      </c>
-      <c r="M87" s="1" t="s">
-        <v>655</v>
-      </c>
-      <c r="N87" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="O87" s="1" t="s">
-        <v>656</v>
-      </c>
-      <c r="P87" s="1" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="88" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:16" ht="14.45" customHeight="true">
       <c r="A88" s="1" t="s">
-        <v>658</v>
+        <v>783</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>129</v>
+        <v>665</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="H88" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>516</v>
+        <v>19</v>
       </c>
       <c r="J88" s="1" t="b">
         <v>0</v>
@@ -6643,27 +6825,45 @@
         <v>716</v>
       </c>
       <c r="L88" s="1" t="s">
-        <v>645</v>
+        <v>668</v>
       </c>
       <c r="M88" s="1" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="89" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>670</v>
+      </c>
+      <c r="O88" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="P88" s="1" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" ht="14.45" customHeight="true">
       <c r="A89" s="1" t="s">
-        <v>698</v>
+        <v>673</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>697</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>705</v>
+        <v>674</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>15</v>
+        <v>109</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="J89" s="1" t="b">
         <v>0</v>
@@ -6671,104 +6871,28 @@
       <c r="K89" s="1" t="s">
         <v>716</v>
       </c>
-    </row>
-    <row r="90" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="1" t="s">
-        <v>664</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>663</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E90" s="1" t="s">
-        <v>665</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>666</v>
-      </c>
-      <c r="G90" s="1" t="s">
-        <v>667</v>
-      </c>
-      <c r="H90" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I90" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J90" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="K90" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="L90" s="1" t="s">
-        <v>668</v>
-      </c>
-      <c r="M90" s="1" t="s">
-        <v>669</v>
-      </c>
-      <c r="N90" s="1" t="s">
-        <v>670</v>
-      </c>
-      <c r="O90" s="1" t="s">
-        <v>671</v>
-      </c>
-      <c r="P90" s="1" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="91" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="1" t="s">
-        <v>673</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>674</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>675</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>676</v>
-      </c>
-      <c r="G91" s="1" t="s">
-        <v>677</v>
-      </c>
-      <c r="H91" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I91" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J91" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="K91" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="L91" s="1" t="s">
+      <c r="L89" s="1" t="s">
         <v>678</v>
       </c>
-      <c r="M91" s="1" t="s">
+      <c r="M89" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="N91" s="1" t="s">
+      <c r="N89" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="O91" s="1" t="s">
+      <c r="O89" s="1" t="s">
         <v>681</v>
       </c>
-      <c r="P91" s="1" t="s">
+      <c r="P89" s="1" t="s">
         <v>682</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>784</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 

</xml_diff>